<commit_message>
More accruals and excel file correction
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/CLOEb.ST.xlsx
+++ b/data/stx_xlsx/CLOEb.ST.xlsx
@@ -11806,21 +11806,39 @@
       <c r="M54" s="17">
         <v>1597.82</v>
       </c>
-      <c r="N54" s="18"/>
-      <c r="O54" s="18"/>
+      <c r="N54" s="23">
+        <f t="shared" ref="N54:O54" si="1">SUM(N55,N57,N59,N53)</f>
+        <v>1564.48</v>
+      </c>
+      <c r="O54" s="23">
+        <f t="shared" si="1"/>
+        <v>1379.06</v>
+      </c>
       <c r="P54" s="17">
         <v>1143.64</v>
       </c>
       <c r="Q54" s="17">
         <v>1143.64</v>
       </c>
-      <c r="R54" s="18"/>
-      <c r="S54" s="18"/>
-      <c r="T54" s="17">
+      <c r="R54" s="23">
+        <f t="shared" ref="R54:S54" si="2">SUM(R53,R55:R59)</f>
+        <v>357</v>
+      </c>
+      <c r="S54" s="23">
+        <f t="shared" si="2"/>
+        <v>374.34</v>
+      </c>
+      <c r="T54" s="23">
         <v>389.4</v>
       </c>
-      <c r="U54" s="18"/>
-      <c r="V54" s="18"/>
+      <c r="U54" s="23">
+        <f t="shared" ref="U54:V54" si="3">SUM(U53,U55:U59)</f>
+        <v>316.21</v>
+      </c>
+      <c r="V54" s="23">
+        <f t="shared" si="3"/>
+        <v>251.46</v>
+      </c>
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="16" t="s">
@@ -13471,23 +13489,23 @@
         <v>257</v>
       </c>
       <c r="B91" s="18">
-        <f t="shared" ref="B91:F91" si="1">B90+B92-B94+B95</f>
+        <f t="shared" ref="B91:F91" si="4">B90+B92-B94+B95</f>
         <v>159.64</v>
       </c>
       <c r="C91" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>153.19</v>
       </c>
       <c r="D91" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>149</v>
       </c>
       <c r="E91" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>139.3</v>
       </c>
       <c r="F91" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>146.14</v>
       </c>
       <c r="G91" s="18">

</xml_diff>